<commit_message>
Add system instructions + updated demo datasets
- C365 agent + assistant system instructions (c365_knowledge/)
- Edco system instructions + updated demo catalog/client history
- Emma system instructions + updated parts catalog/model mapping

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/emma_knowledge/Emma_Demo_Model_Mapping.xlsx
+++ b/emma_knowledge/Emma_Demo_Model_Mapping.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model Mapping" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Model Mapping'!$A$1:$F$201</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -28,24 +26,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
-        <bgColor rgb="001F4E79"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -68,8 +57,8 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -438,14 +427,6 @@
   </sheetPr>
   <dimension ref="A1:F201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -6880,7 +6861,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F201"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>